<commit_message>
Fixed incorrect wheat. Fixed missing scenarios. Modified dataprep function to print lu being skipped
</commit_message>
<xml_diff>
--- a/data/crops/FAO_GAEZ/crops_file_index.xlsx
+++ b/data/crops/FAO_GAEZ/crops_file_index.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/FAO_GAEZ/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F1E3413AAE31921FD23EBBD24029C062B3104491" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B124D74-2ED3-4F74-99FC-2CB373295DD6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -679,8 +673,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -718,48 +712,36 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf/>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:J54" totalsRowShown="0">
-  <autoFilter ref="A1:J54" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="annual"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:J54" totalsRowShown="0">
+  <autoFilter ref="A1:J54"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="crop_name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="crop_practice_string"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="crop_type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="irrigation_practice"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="filename"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="filepath"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="crop_code"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tech_code"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="technology"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="lu_file"/>
+    <tableColumn id="1" name="crop_name" dataDxfId="0"/>
+    <tableColumn id="2" name="crop_practice_string" dataDxfId="0"/>
+    <tableColumn id="3" name="crop_type" dataDxfId="0"/>
+    <tableColumn id="4" name="irrigation_practice" dataDxfId="0"/>
+    <tableColumn id="5" name="filename" dataDxfId="0"/>
+    <tableColumn id="6" name="filepath" dataDxfId="0"/>
+    <tableColumn id="7" name="crop_code" dataDxfId="0"/>
+    <tableColumn id="8" name="tech_code" dataDxfId="0"/>
+    <tableColumn id="9" name="technology" dataDxfId="0"/>
+    <tableColumn id="10" name="lu_file" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -797,7 +779,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -831,7 +813,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -866,10 +847,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1042,11 +1022,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J54"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1078,7 +1058,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1110,7 +1090,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1142,7 +1122,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1174,7 +1154,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -1206,7 +1186,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" s="1" t="s">
         <v>32</v>
       </c>
@@ -1238,7 +1218,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -1270,7 +1250,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1302,7 +1282,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
@@ -1334,7 +1314,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -1366,7 +1346,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="1" t="s">
         <v>53</v>
       </c>
@@ -1398,7 +1378,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="1" t="s">
         <v>58</v>
       </c>
@@ -1430,7 +1410,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="1" t="s">
         <v>58</v>
       </c>
@@ -1462,7 +1442,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10">
       <c r="A14" s="1" t="s">
         <v>64</v>
       </c>
@@ -1494,7 +1474,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10">
       <c r="A15" s="1" t="s">
         <v>69</v>
       </c>
@@ -1526,7 +1506,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10">
       <c r="A16" s="1" t="s">
         <v>74</v>
       </c>
@@ -1558,7 +1538,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1590,7 +1570,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10">
       <c r="A18" s="1" t="s">
         <v>84</v>
       </c>
@@ -1622,7 +1602,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10">
       <c r="A19" s="1" t="s">
         <v>89</v>
       </c>
@@ -1654,7 +1634,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
         <v>94</v>
       </c>
@@ -1686,7 +1666,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10">
       <c r="A21" s="1" t="s">
         <v>94</v>
       </c>
@@ -1718,7 +1698,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1750,7 +1730,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -1782,7 +1762,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10">
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1814,7 +1794,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10">
       <c r="A25" s="1" t="s">
         <v>37</v>
       </c>
@@ -1846,7 +1826,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
@@ -1878,7 +1858,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10">
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
@@ -1910,7 +1890,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10">
       <c r="A28" s="1" t="s">
         <v>58</v>
       </c>
@@ -1942,7 +1922,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10">
       <c r="A29" s="1" t="s">
         <v>69</v>
       </c>
@@ -1974,7 +1954,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -2006,7 +1986,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
         <v>74</v>
       </c>
@@ -2038,7 +2018,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
         <v>79</v>
       </c>
@@ -2070,7 +2050,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10">
       <c r="A33" s="1" t="s">
         <v>84</v>
       </c>
@@ -2102,7 +2082,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10">
       <c r="A34" s="1" t="s">
         <v>89</v>
       </c>
@@ -2134,7 +2114,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10">
       <c r="A35" s="1" t="s">
         <v>94</v>
       </c>
@@ -2166,7 +2146,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10">
       <c r="A36" s="1" t="s">
         <v>144</v>
       </c>
@@ -2198,7 +2178,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10">
       <c r="A37" s="1" t="s">
         <v>144</v>
       </c>
@@ -2230,7 +2210,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10">
       <c r="A38" s="1" t="s">
         <v>53</v>
       </c>
@@ -2262,7 +2242,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10">
       <c r="A39" s="1" t="s">
         <v>153</v>
       </c>
@@ -2294,7 +2274,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10">
       <c r="A40" s="1" t="s">
         <v>153</v>
       </c>
@@ -2326,7 +2306,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10">
       <c r="A41" s="1" t="s">
         <v>162</v>
       </c>
@@ -2358,7 +2338,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10">
       <c r="A42" s="1" t="s">
         <v>162</v>
       </c>
@@ -2390,7 +2370,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10">
       <c r="A43" s="1" t="s">
         <v>170</v>
       </c>
@@ -2422,7 +2402,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10">
       <c r="A44" s="1" t="s">
         <v>170</v>
       </c>
@@ -2454,7 +2434,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10">
       <c r="A45" s="1" t="s">
         <v>178</v>
       </c>
@@ -2486,7 +2466,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10">
       <c r="A46" s="1" t="s">
         <v>178</v>
       </c>
@@ -2518,7 +2498,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10">
       <c r="A47" s="1" t="s">
         <v>186</v>
       </c>
@@ -2550,7 +2530,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10">
       <c r="A48" s="1" t="s">
         <v>186</v>
       </c>
@@ -2582,7 +2562,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10">
       <c r="A49" s="1" t="s">
         <v>194</v>
       </c>
@@ -2614,7 +2594,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10">
       <c r="A50" s="1" t="s">
         <v>194</v>
       </c>
@@ -2646,7 +2626,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10">
       <c r="A51" s="1" t="s">
         <v>202</v>
       </c>
@@ -2678,7 +2658,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10">
       <c r="A52" s="1" t="s">
         <v>202</v>
       </c>
@@ -2710,7 +2690,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10">
       <c r="A53" s="1" t="s">
         <v>210</v>
       </c>
@@ -2742,7 +2722,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10">
       <c r="A54" s="1" t="s">
         <v>210</v>
       </c>

</xml_diff>

<commit_message>
rerun soc country averages, updated crop land use files inventory
</commit_message>
<xml_diff>
--- a/data/crops/FAO_GAEZ/crops_file_index.xlsx
+++ b/data/crops/FAO_GAEZ/crops_file_index.xlsx
@@ -1,15 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/FAO_GAEZ/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_F0EC413AAE31921FD23EBBD24029C062E31A7711" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0988B5B-5556-4080-BCC7-60CFC0DFFB83}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -673,8 +692,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -712,36 +731,42 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf/>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:J54" totalsRowShown="0">
-  <autoFilter ref="A1:J54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:J54" totalsRowShown="0">
+  <autoFilter ref="A1:J54" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" name="crop_name" dataDxfId="0"/>
-    <tableColumn id="2" name="crop_practice_string" dataDxfId="0"/>
-    <tableColumn id="3" name="crop_type" dataDxfId="0"/>
-    <tableColumn id="4" name="irrigation_practice" dataDxfId="0"/>
-    <tableColumn id="5" name="filename" dataDxfId="0"/>
-    <tableColumn id="6" name="filepath" dataDxfId="0"/>
-    <tableColumn id="7" name="crop_code" dataDxfId="0"/>
-    <tableColumn id="8" name="tech_code" dataDxfId="0"/>
-    <tableColumn id="9" name="technology" dataDxfId="0"/>
-    <tableColumn id="10" name="lu_file" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="crop_name"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="crop_practice_string"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="crop_type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="irrigation_practice"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="filename"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="filepath"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="crop_code"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tech_code"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="technology"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="lu_file"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -779,7 +804,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -813,6 +838,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -847,9 +873,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1022,11 +1049,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J54"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1058,7 +1085,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1090,7 +1117,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1122,7 +1149,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1154,7 +1181,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -1186,7 +1213,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>32</v>
       </c>
@@ -1218,7 +1245,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -1250,7 +1277,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1282,7 +1309,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
@@ -1314,7 +1341,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -1346,7 +1373,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>53</v>
       </c>
@@ -1378,7 +1405,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>58</v>
       </c>
@@ -1410,7 +1437,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>58</v>
       </c>
@@ -1442,7 +1469,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>64</v>
       </c>
@@ -1474,7 +1501,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>69</v>
       </c>
@@ -1506,7 +1533,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>74</v>
       </c>
@@ -1538,7 +1565,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1570,7 +1597,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>84</v>
       </c>
@@ -1602,7 +1629,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>89</v>
       </c>
@@ -1634,7 +1661,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>94</v>
       </c>
@@ -1666,7 +1693,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>94</v>
       </c>
@@ -1698,7 +1725,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1730,7 +1757,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -1762,7 +1789,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1794,7 +1821,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>37</v>
       </c>
@@ -1826,7 +1853,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
@@ -1858,7 +1885,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
@@ -1890,7 +1917,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>58</v>
       </c>
@@ -1922,7 +1949,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>69</v>
       </c>
@@ -1954,7 +1981,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1986,7 +2013,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>74</v>
       </c>
@@ -2018,7 +2045,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>79</v>
       </c>
@@ -2050,7 +2077,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>84</v>
       </c>
@@ -2082,7 +2109,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>89</v>
       </c>
@@ -2114,7 +2141,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>94</v>
       </c>
@@ -2146,7 +2173,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>144</v>
       </c>
@@ -2178,7 +2205,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>144</v>
       </c>
@@ -2210,7 +2237,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>53</v>
       </c>
@@ -2242,7 +2269,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>153</v>
       </c>
@@ -2274,7 +2301,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>153</v>
       </c>
@@ -2306,7 +2333,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>162</v>
       </c>
@@ -2338,7 +2365,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>162</v>
       </c>
@@ -2370,7 +2397,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>170</v>
       </c>
@@ -2402,7 +2429,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>170</v>
       </c>
@@ -2434,7 +2461,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>178</v>
       </c>
@@ -2466,7 +2493,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>178</v>
       </c>
@@ -2498,7 +2525,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>186</v>
       </c>
@@ -2530,7 +2557,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>186</v>
       </c>
@@ -2562,7 +2589,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>194</v>
       </c>
@@ -2594,7 +2621,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>194</v>
       </c>
@@ -2626,7 +2653,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>202</v>
       </c>
@@ -2658,7 +2685,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>202</v>
       </c>
@@ -2690,7 +2717,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>210</v>
       </c>
@@ -2722,7 +2749,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>210</v>
       </c>

</xml_diff>